<commit_message>
DF makes changes - "Poland Update"
</commit_message>
<xml_diff>
--- a/reading_wines/wine_company_inventory.xlsx
+++ b/reading_wines/wine_company_inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://saintkentigern-my.sharepoint.com/personal/h_c_sutton_student_saintkentigern_com/Documents/Desktop/COMSCI 2026/1_g1t/UI Layout 5/reading_wines/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B58DFD4-4EC2-4427-9212-C147F6C009FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{5B58DFD4-4EC2-4427-9212-C147F6C009FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9DA312A-9FC6-427B-B553-59D90BB95A71}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4310" uniqueCount="777">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4311" uniqueCount="778">
   <si>
     <t>Wine ID</t>
   </si>
@@ -2365,6 +2365,9 @@
   </si>
   <si>
     <t>TOTAL</t>
+  </si>
+  <si>
+    <t>Poland</t>
   </si>
 </sst>
 </file>
@@ -2438,7 +2441,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="WineInventoryTable" displayName="WineInventoryTable" ref="A1:AD251" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="WineInventoryTable" displayName="WineInventoryTable" ref="A1:AD252" totalsRowShown="0">
   <tableColumns count="30">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Wine ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Wine Name"/>
@@ -2681,7 +2684,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AD251"/>
+  <dimension ref="A1:AD252"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -20885,7 +20888,7 @@
         <v>67.489999999999995</v>
       </c>
       <c r="R194" s="4">
-        <f t="shared" ref="R194:R257" si="6">IFERROR((P194-Q194)/P194,0)</f>
+        <f t="shared" ref="R194:R251" si="6">IFERROR((P194-Q194)/P194,0)</f>
         <v>0.39595453324979868</v>
       </c>
       <c r="S194">
@@ -26282,6 +26285,11 @@
       </c>
       <c r="AD251">
         <v>2038</v>
+      </c>
+    </row>
+    <row r="252" spans="1:30">
+      <c r="D252" t="s">
+        <v>777</v>
       </c>
     </row>
   </sheetData>
@@ -26317,7 +26325,7 @@
         <v>49</v>
       </c>
       <c r="B2">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A2)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A2)</f>
         <v>65</v>
       </c>
       <c r="C2" s="4">
@@ -26330,7 +26338,7 @@
         <v>33</v>
       </c>
       <c r="B3">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A3)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A3)</f>
         <v>45</v>
       </c>
       <c r="C3" s="4">
@@ -26343,7 +26351,7 @@
         <v>152</v>
       </c>
       <c r="B4">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A4)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A4)</f>
         <v>32</v>
       </c>
       <c r="C4" s="4">
@@ -26356,7 +26364,7 @@
         <v>105</v>
       </c>
       <c r="B5">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A5)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A5)</f>
         <v>25</v>
       </c>
       <c r="C5" s="4">
@@ -26369,7 +26377,7 @@
         <v>110</v>
       </c>
       <c r="B6">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A6)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A6)</f>
         <v>20</v>
       </c>
       <c r="C6" s="4">
@@ -26382,7 +26390,7 @@
         <v>160</v>
       </c>
       <c r="B7">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A7)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A7)</f>
         <v>14</v>
       </c>
       <c r="C7" s="4">
@@ -26395,7 +26403,7 @@
         <v>227</v>
       </c>
       <c r="B8">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A8)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A8)</f>
         <v>9</v>
       </c>
       <c r="C8" s="4">
@@ -26408,7 +26416,7 @@
         <v>129</v>
       </c>
       <c r="B9">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A9)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A9)</f>
         <v>7</v>
       </c>
       <c r="C9" s="4">
@@ -26421,7 +26429,7 @@
         <v>116</v>
       </c>
       <c r="B10">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A10)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A10)</f>
         <v>6</v>
       </c>
       <c r="C10" s="4">
@@ -26434,7 +26442,7 @@
         <v>59</v>
       </c>
       <c r="B11">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A11)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A11)</f>
         <v>5</v>
       </c>
       <c r="C11" s="4">
@@ -26447,7 +26455,7 @@
         <v>98</v>
       </c>
       <c r="B12">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A12)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A12)</f>
         <v>4</v>
       </c>
       <c r="C12" s="4">
@@ -26460,7 +26468,7 @@
         <v>384</v>
       </c>
       <c r="B13">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A13)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A13)</f>
         <v>3</v>
       </c>
       <c r="C13" s="4">
@@ -26473,7 +26481,7 @@
         <v>355</v>
       </c>
       <c r="B14">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A14)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A14)</f>
         <v>2</v>
       </c>
       <c r="C14" s="4">
@@ -26486,7 +26494,7 @@
         <v>609</v>
       </c>
       <c r="B15">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A15)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A15)</f>
         <v>2</v>
       </c>
       <c r="C15" s="4">
@@ -26499,7 +26507,7 @@
         <v>312</v>
       </c>
       <c r="B16">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A16)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A16)</f>
         <v>2</v>
       </c>
       <c r="C16" s="4">
@@ -26512,7 +26520,7 @@
         <v>253</v>
       </c>
       <c r="B17">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A17)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A17)</f>
         <v>1</v>
       </c>
       <c r="C17" s="4">
@@ -26525,7 +26533,7 @@
         <v>507</v>
       </c>
       <c r="B18">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A18)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A18)</f>
         <v>1</v>
       </c>
       <c r="C18" s="4">
@@ -26538,7 +26546,7 @@
         <v>136</v>
       </c>
       <c r="B19">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A19)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A19)</f>
         <v>1</v>
       </c>
       <c r="C19" s="4">
@@ -26551,7 +26559,7 @@
         <v>142</v>
       </c>
       <c r="B20">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A20)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A20)</f>
         <v>1</v>
       </c>
       <c r="C20" s="4">
@@ -26564,7 +26572,7 @@
         <v>491</v>
       </c>
       <c r="B21">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A21)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A21)</f>
         <v>1</v>
       </c>
       <c r="C21" s="4">
@@ -26577,7 +26585,7 @@
         <v>342</v>
       </c>
       <c r="B22">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A22)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A22)</f>
         <v>1</v>
       </c>
       <c r="C22" s="4">
@@ -26590,7 +26598,7 @@
         <v>618</v>
       </c>
       <c r="B23">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A23)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A23)</f>
         <v>1</v>
       </c>
       <c r="C23" s="4">
@@ -26603,7 +26611,7 @@
         <v>689</v>
       </c>
       <c r="B24">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A24)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A24)</f>
         <v>1</v>
       </c>
       <c r="C24" s="4">
@@ -26616,7 +26624,7 @@
         <v>419</v>
       </c>
       <c r="B25">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$251,A25)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A25)</f>
         <v>1</v>
       </c>
       <c r="C25" s="4">

</xml_diff>

<commit_message>
Read Me Change Update
</commit_message>
<xml_diff>
--- a/reading_wines/wine_company_inventory.xlsx
+++ b/reading_wines/wine_company_inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://saintkentigern-my.sharepoint.com/personal/h_c_sutton_student_saintkentigern_com/Documents/Desktop/COMSCI 2026/1_g1t/UI Layout 5/reading_wines/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{5B58DFD4-4EC2-4427-9212-C147F6C009FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9DA312A-9FC6-427B-B553-59D90BB95A71}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{5B58DFD4-4EC2-4427-9212-C147F6C009FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8399E3A-F394-4739-8E0E-5BAF8F23344C}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4311" uniqueCount="778">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4310" uniqueCount="777">
   <si>
     <t>Wine ID</t>
   </si>
@@ -2365,9 +2365,6 @@
   </si>
   <si>
     <t>TOTAL</t>
-  </si>
-  <si>
-    <t>Poland</t>
   </si>
 </sst>
 </file>
@@ -2378,7 +2375,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -2387,6 +2384,12 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFF7E8BA"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -2412,10 +2415,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2423,8 +2427,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2440,8 +2446,12 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="WineInventoryTable" displayName="WineInventoryTable" ref="A1:AD252" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="WineInventoryTable" displayName="WineInventoryTable" ref="A1:AD257" totalsRowShown="0">
   <tableColumns count="30">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Wine ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Wine Name"/>
@@ -26288,9 +26298,7 @@
       </c>
     </row>
     <row r="252" spans="1:30">
-      <c r="D252" t="s">
-        <v>777</v>
-      </c>
+      <c r="D252" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -26325,7 +26333,7 @@
         <v>49</v>
       </c>
       <c r="B2">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A2)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A2)</f>
         <v>65</v>
       </c>
       <c r="C2" s="4">
@@ -26338,7 +26346,7 @@
         <v>33</v>
       </c>
       <c r="B3">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A3)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A3)</f>
         <v>45</v>
       </c>
       <c r="C3" s="4">
@@ -26351,7 +26359,7 @@
         <v>152</v>
       </c>
       <c r="B4">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A4)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A4)</f>
         <v>32</v>
       </c>
       <c r="C4" s="4">
@@ -26364,7 +26372,7 @@
         <v>105</v>
       </c>
       <c r="B5">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A5)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A5)</f>
         <v>25</v>
       </c>
       <c r="C5" s="4">
@@ -26377,7 +26385,7 @@
         <v>110</v>
       </c>
       <c r="B6">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A6)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A6)</f>
         <v>20</v>
       </c>
       <c r="C6" s="4">
@@ -26390,7 +26398,7 @@
         <v>160</v>
       </c>
       <c r="B7">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A7)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A7)</f>
         <v>14</v>
       </c>
       <c r="C7" s="4">
@@ -26403,7 +26411,7 @@
         <v>227</v>
       </c>
       <c r="B8">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A8)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A8)</f>
         <v>9</v>
       </c>
       <c r="C8" s="4">
@@ -26416,7 +26424,7 @@
         <v>129</v>
       </c>
       <c r="B9">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A9)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A9)</f>
         <v>7</v>
       </c>
       <c r="C9" s="4">
@@ -26429,7 +26437,7 @@
         <v>116</v>
       </c>
       <c r="B10">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A10)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A10)</f>
         <v>6</v>
       </c>
       <c r="C10" s="4">
@@ -26442,7 +26450,7 @@
         <v>59</v>
       </c>
       <c r="B11">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A11)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A11)</f>
         <v>5</v>
       </c>
       <c r="C11" s="4">
@@ -26455,7 +26463,7 @@
         <v>98</v>
       </c>
       <c r="B12">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A12)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A12)</f>
         <v>4</v>
       </c>
       <c r="C12" s="4">
@@ -26468,7 +26476,7 @@
         <v>384</v>
       </c>
       <c r="B13">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A13)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A13)</f>
         <v>3</v>
       </c>
       <c r="C13" s="4">
@@ -26481,7 +26489,7 @@
         <v>355</v>
       </c>
       <c r="B14">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A14)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A14)</f>
         <v>2</v>
       </c>
       <c r="C14" s="4">
@@ -26494,7 +26502,7 @@
         <v>609</v>
       </c>
       <c r="B15">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A15)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A15)</f>
         <v>2</v>
       </c>
       <c r="C15" s="4">
@@ -26507,7 +26515,7 @@
         <v>312</v>
       </c>
       <c r="B16">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A16)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A16)</f>
         <v>2</v>
       </c>
       <c r="C16" s="4">
@@ -26520,7 +26528,7 @@
         <v>253</v>
       </c>
       <c r="B17">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A17)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A17)</f>
         <v>1</v>
       </c>
       <c r="C17" s="4">
@@ -26533,7 +26541,7 @@
         <v>507</v>
       </c>
       <c r="B18">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A18)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A18)</f>
         <v>1</v>
       </c>
       <c r="C18" s="4">
@@ -26546,7 +26554,7 @@
         <v>136</v>
       </c>
       <c r="B19">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A19)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A19)</f>
         <v>1</v>
       </c>
       <c r="C19" s="4">
@@ -26559,7 +26567,7 @@
         <v>142</v>
       </c>
       <c r="B20">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A20)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A20)</f>
         <v>1</v>
       </c>
       <c r="C20" s="4">
@@ -26572,7 +26580,7 @@
         <v>491</v>
       </c>
       <c r="B21">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A21)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A21)</f>
         <v>1</v>
       </c>
       <c r="C21" s="4">
@@ -26585,7 +26593,7 @@
         <v>342</v>
       </c>
       <c r="B22">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A22)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A22)</f>
         <v>1</v>
       </c>
       <c r="C22" s="4">
@@ -26598,7 +26606,7 @@
         <v>618</v>
       </c>
       <c r="B23">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A23)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A23)</f>
         <v>1</v>
       </c>
       <c r="C23" s="4">
@@ -26611,7 +26619,7 @@
         <v>689</v>
       </c>
       <c r="B24">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A24)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A24)</f>
         <v>1</v>
       </c>
       <c r="C24" s="4">
@@ -26624,7 +26632,7 @@
         <v>419</v>
       </c>
       <c r="B25">
-        <f>COUNTIF('Wine Inventory'!$D$2:$D$252,A25)</f>
+        <f>COUNTIF('Wine Inventory'!$D$2:$D$257,A25)</f>
         <v>1</v>
       </c>
       <c r="C25" s="4">

</xml_diff>